<commit_message>
Aggiunge import massivo tipi evento e dettagli da Excel.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Voci impostazioni.xlsx
+++ b/Voci impostazioni.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\App_mie\CROSS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{519D7E9A-29A7-47A3-BF5B-93437CB7CB74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{828A467C-1E04-46E1-A77C-631B89687B27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -159,9 +159,6 @@
     <t>MORSO</t>
   </si>
   <si>
-    <t>ZZA</t>
-  </si>
-  <si>
     <t>RESPIRATORIA</t>
   </si>
   <si>
@@ -502,6 +499,9 @@
   </si>
   <si>
     <t>ALTRO NON CLASSIFICA</t>
+  </si>
+  <si>
+    <t>ALTRO NON NOTO</t>
   </si>
 </sst>
 </file>
@@ -1026,48 +1026,48 @@
         <v>43</v>
       </c>
       <c r="W2" s="4" t="s">
-        <v>44</v>
+        <v>158</v>
       </c>
     </row>
     <row r="3" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="H3" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="I3" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="J3" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="K3" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="L3" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="K3" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="L3" s="3" t="s">
+      <c r="M3" s="3" t="s">
         <v>55</v>
-      </c>
-      <c r="M3" s="3" t="s">
-        <v>56</v>
       </c>
       <c r="N3" s="3" t="s">
         <v>2</v>
@@ -1076,222 +1076,222 @@
         <v>2</v>
       </c>
       <c r="P3" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q3" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="Q3" s="3" t="s">
+      <c r="R3" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="R3" s="3" t="s">
+      <c r="S3" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="S3" s="3" t="s">
+      <c r="T3" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="T3" s="3" t="s">
+      <c r="U3" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="U3" s="3" t="s">
+      <c r="V3" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="V3" s="3" t="s">
+      <c r="W3" s="4" t="s">
         <v>63</v>
-      </c>
-      <c r="W3" s="4" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="4" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="F4" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="G4" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="H4" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="I4" s="3" t="s">
         <v>72</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>73</v>
       </c>
       <c r="J4" s="3" t="s">
         <v>33</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="L4" s="3" t="s">
         <v>32</v>
       </c>
       <c r="M4" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="N4" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="N4" s="3" t="s">
+      <c r="O4" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="P4" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="O4" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="P4" s="3" t="s">
+      <c r="Q4" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="Q4" s="3" t="s">
+      <c r="R4" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="R4" s="3" t="s">
+      <c r="S4" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="S4" s="3" t="s">
+      <c r="T4" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="T4" s="3" t="s">
+      <c r="U4" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="U4" s="3" t="s">
-        <v>82</v>
-      </c>
       <c r="V4" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="W4" s="4"/>
     </row>
     <row r="5" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="F5" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="G5" s="3" t="s">
         <v>88</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>89</v>
       </c>
       <c r="H5" s="3" t="s">
         <v>6</v>
       </c>
       <c r="I5" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="K5" s="3" t="s">
         <v>90</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="K5" s="3" t="s">
-        <v>91</v>
       </c>
       <c r="L5" s="3" t="s">
         <v>33</v>
       </c>
       <c r="M5" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="N5" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="N5" s="3" t="s">
+      <c r="O5" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="O5" s="3" t="s">
+      <c r="P5" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="P5" s="3" t="s">
+      <c r="Q5" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="Q5" s="3" t="s">
+      <c r="R5" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="S5" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="R5" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="S5" s="3" t="s">
+      <c r="T5" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="T5" s="3" t="s">
+      <c r="U5" s="3" t="s">
         <v>98</v>
-      </c>
-      <c r="U5" s="3" t="s">
-        <v>99</v>
       </c>
       <c r="V5" s="3"/>
       <c r="W5" s="4"/>
     </row>
     <row r="6" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="C6" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="D6" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="E6" s="3" t="s">
+      <c r="F6" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="G6" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="H6" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="H6" s="3" t="s">
+      <c r="I6" s="3" t="s">
         <v>106</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>107</v>
       </c>
       <c r="J6" s="3" t="s">
         <v>34</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="M6" s="3"/>
       <c r="N6" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="O6" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="P6" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="P6" s="3" t="s">
+      <c r="Q6" s="3" t="s">
         <v>110</v>
-      </c>
-      <c r="Q6" s="3" t="s">
-        <v>111</v>
       </c>
       <c r="R6" s="3"/>
       <c r="S6" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="T6" s="3" t="s">
         <v>112</v>
-      </c>
-      <c r="T6" s="3" t="s">
-        <v>113</v>
       </c>
       <c r="U6" s="3"/>
       <c r="V6" s="3"/>
@@ -1299,51 +1299,51 @@
     </row>
     <row r="7" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>115</v>
-      </c>
       <c r="C7" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F7" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="G7" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="H7" s="3" t="s">
         <v>117</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>118</v>
       </c>
       <c r="I7" s="3"/>
       <c r="J7" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="K7" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="K7" s="3" t="s">
+      <c r="L7" s="3" t="s">
         <v>120</v>
-      </c>
-      <c r="L7" s="3" t="s">
-        <v>121</v>
       </c>
       <c r="M7" s="3"/>
       <c r="N7" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="O7" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="P7" s="3" t="s">
         <v>122</v>
-      </c>
-      <c r="P7" s="3" t="s">
-        <v>123</v>
       </c>
       <c r="Q7" s="3"/>
       <c r="R7" s="3"/>
       <c r="S7" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="T7" s="3"/>
       <c r="U7" s="3"/>
@@ -1352,47 +1352,47 @@
     </row>
     <row r="8" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>125</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>126</v>
       </c>
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
       <c r="F8" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I8" s="3"/>
       <c r="J8" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="M8" s="3"/>
       <c r="N8" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="O8" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="O8" s="3" t="s">
+      <c r="P8" s="3" t="s">
         <v>130</v>
-      </c>
-      <c r="P8" s="3" t="s">
-        <v>131</v>
       </c>
       <c r="Q8" s="3"/>
       <c r="R8" s="3"/>
       <c r="S8" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="T8" s="3"/>
       <c r="U8" s="3"/>
@@ -1401,39 +1401,39 @@
     </row>
     <row r="9" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>133</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>134</v>
       </c>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
       <c r="F9" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
       <c r="J9" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="K9" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="L9" s="3" t="s">
         <v>136</v>
-      </c>
-      <c r="K9" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="L9" s="3" t="s">
-        <v>137</v>
       </c>
       <c r="M9" s="3"/>
       <c r="N9" s="3"/>
       <c r="O9" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="P9" s="3"/>
       <c r="Q9" s="3"/>
       <c r="R9" s="3"/>
       <c r="S9" s="3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="T9" s="3"/>
       <c r="U9" s="3"/>
@@ -1442,26 +1442,26 @@
     </row>
     <row r="10" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>140</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>141</v>
       </c>
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
       <c r="F10" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
       <c r="J10" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="K10" s="3"/>
       <c r="L10" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="M10" s="3"/>
       <c r="N10" s="3"/>
@@ -1470,7 +1470,7 @@
       <c r="Q10" s="3"/>
       <c r="R10" s="3"/>
       <c r="S10" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="T10" s="3"/>
       <c r="U10" s="3"/>
@@ -1479,10 +1479,10 @@
     </row>
     <row r="11" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>143</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>144</v>
       </c>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
@@ -1501,7 +1501,7 @@
       <c r="Q11" s="3"/>
       <c r="R11" s="3"/>
       <c r="S11" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="T11" s="3"/>
       <c r="U11" s="3"/>
@@ -1510,10 +1510,10 @@
     </row>
     <row r="12" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
@@ -1532,7 +1532,7 @@
       <c r="Q12" s="3"/>
       <c r="R12" s="3"/>
       <c r="S12" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="T12" s="3"/>
       <c r="U12" s="3"/>
@@ -1541,10 +1541,10 @@
     </row>
     <row r="13" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="B13" s="3" t="s">
         <v>148</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>149</v>
       </c>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
@@ -1563,7 +1563,7 @@
       <c r="Q13" s="3"/>
       <c r="R13" s="3"/>
       <c r="S13" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="T13" s="3"/>
       <c r="U13" s="3"/>
@@ -1572,10 +1572,10 @@
     </row>
     <row r="14" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="B14" s="3" t="s">
         <v>151</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>152</v>
       </c>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
@@ -1594,7 +1594,7 @@
       <c r="Q14" s="3"/>
       <c r="R14" s="3"/>
       <c r="S14" s="3" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="T14" s="3"/>
       <c r="U14" s="3"/>
@@ -1603,10 +1603,10 @@
     </row>
     <row r="15" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="B15" s="3" t="s">
         <v>154</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>155</v>
       </c>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
@@ -1632,10 +1632,10 @@
     </row>
     <row r="16" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
@@ -1661,7 +1661,7 @@
     </row>
     <row r="17" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -1688,7 +1688,7 @@
     </row>
     <row r="18" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>

</xml_diff>

<commit_message>
v1.5: dashboard operativa, PMA, Telegram missione e integrazione PMApp.
- Dashboard: colonne E/M/T, eventi terminati, esiti missione e layout missioni

- PMA in impostazioni/mappa; ospedali destinazione includono i PMA creati

- Telegram: messaggio missione con data, ID, colore M e campi evento richiesti

- Header: brand CROSS, pulsanti + Evento e Reset vista dopo sync

- Evento: chiamante, luogo, meteo; MSA/MSB; SOREU; sync PMApp su DIRETTO H

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Voci impostazioni.xlsx
+++ b/Voci impostazioni.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\App_mie\CROSS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{828A467C-1E04-46E1-A77C-631B89687B27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8523F798-3645-45B1-B066-8A9AC402332C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Eventi e dettagli" sheetId="1" r:id="rId1"/>
+    <sheet name="Luoghi e dettagli" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="279">
   <si>
     <t>MEDICO ACUTO</t>
   </si>
@@ -502,6 +503,366 @@
   </si>
   <si>
     <t>ALTRO NON NOTO</t>
+  </si>
+  <si>
+    <t>CASA</t>
+  </si>
+  <si>
+    <t>STRADA</t>
+  </si>
+  <si>
+    <t>UFFICIO LUOGO PUBBLICO</t>
+  </si>
+  <si>
+    <t>IMPIANTO LAVORATIVO</t>
+  </si>
+  <si>
+    <t>IMPIANTO SPORTIVO</t>
+  </si>
+  <si>
+    <t>SCUOLA</t>
+  </si>
+  <si>
+    <t>OSPEDALE</t>
+  </si>
+  <si>
+    <t>ANDRONE</t>
+  </si>
+  <si>
+    <t>AUTOSTRADA/TANG.</t>
+  </si>
+  <si>
+    <t>AEROPORTO LINATE</t>
+  </si>
+  <si>
+    <t>AREA AGRICOLA</t>
+  </si>
+  <si>
+    <t>AUTODROMO</t>
+  </si>
+  <si>
+    <t>CAMPO SPORTIVO</t>
+  </si>
+  <si>
+    <t>AMBULATORIO</t>
+  </si>
+  <si>
+    <t>BOX</t>
+  </si>
+  <si>
+    <t>CAMPO NOMADI</t>
+  </si>
+  <si>
+    <t>AEROPORTO MALPENSA</t>
+  </si>
+  <si>
+    <t>CANTIERE</t>
+  </si>
+  <si>
+    <t>CLASSE</t>
+  </si>
+  <si>
+    <t>INGRESSO</t>
+  </si>
+  <si>
+    <t>CANTINA</t>
+  </si>
+  <si>
+    <t>CARREGGIATA</t>
+  </si>
+  <si>
+    <t>AEROPORTO ORIO</t>
+  </si>
+  <si>
+    <t>IPPODROMO</t>
+  </si>
+  <si>
+    <t>CORTILE</t>
+  </si>
+  <si>
+    <t>PADIGLIONE</t>
+  </si>
+  <si>
+    <t>GIARDINO</t>
+  </si>
+  <si>
+    <t>BAR</t>
+  </si>
+  <si>
+    <t>MOTODROMO</t>
+  </si>
+  <si>
+    <t>INFERMERIA</t>
+  </si>
+  <si>
+    <t>PARCHEGGIO</t>
+  </si>
+  <si>
+    <t>MARCIAPIEDE</t>
+  </si>
+  <si>
+    <t>CAMPO VOLO</t>
+  </si>
+  <si>
+    <t>PALASPORT</t>
+  </si>
+  <si>
+    <t>PORTA CARRAIA</t>
+  </si>
+  <si>
+    <t>PORTINERIA</t>
+  </si>
+  <si>
+    <t>CARCERE*</t>
+  </si>
+  <si>
+    <t>PALESTRA</t>
+  </si>
+  <si>
+    <t>LABORATORIO</t>
+  </si>
+  <si>
+    <t>PPI</t>
+  </si>
+  <si>
+    <t>SCALE</t>
+  </si>
+  <si>
+    <t>CASERMA*</t>
+  </si>
+  <si>
+    <t>MAGAZZINO</t>
+  </si>
+  <si>
+    <t>PISCINA</t>
+  </si>
+  <si>
+    <t>PS</t>
+  </si>
+  <si>
+    <t>SOLAIO</t>
+  </si>
+  <si>
+    <t>PARCO</t>
+  </si>
+  <si>
+    <t>CENTRO ACCOGLIENZA</t>
+  </si>
+  <si>
+    <t>OFFICINA</t>
+  </si>
+  <si>
+    <t>SPALTI PUBBLICO</t>
+  </si>
+  <si>
+    <t>REPARTO</t>
+  </si>
+  <si>
+    <t>ALTRO</t>
+  </si>
+  <si>
+    <t>ROTONDA</t>
+  </si>
+  <si>
+    <t>CENTRO COMMERCIALE</t>
+  </si>
+  <si>
+    <t>UFFICIO</t>
+  </si>
+  <si>
+    <t>SPOGLIATOIO</t>
+  </si>
+  <si>
+    <t>STRADE INTERNE</t>
+  </si>
+  <si>
+    <t>TRATTA EXTRAURBANA</t>
+  </si>
+  <si>
+    <t>CIMITERO</t>
+  </si>
+  <si>
+    <t>STADIO</t>
+  </si>
+  <si>
+    <t>TRATTA URBANA</t>
+  </si>
+  <si>
+    <t>CINEMA/TEATRO/DISCO</t>
+  </si>
+  <si>
+    <t>COMMISSARIATO*</t>
+  </si>
+  <si>
+    <t>FARMACIA</t>
+  </si>
+  <si>
+    <t>LUOGO DI CULTO</t>
+  </si>
+  <si>
+    <t>NEGOZIO</t>
+  </si>
+  <si>
+    <t>ORATORIO</t>
+  </si>
+  <si>
+    <t>PREFETTURA</t>
+  </si>
+  <si>
+    <t>QUESTURA*</t>
+  </si>
+  <si>
+    <t>RISTORANTE</t>
+  </si>
+  <si>
+    <t>STRUT. ALBERGHIERA</t>
+  </si>
+  <si>
+    <t>SUPERMERCATO</t>
+  </si>
+  <si>
+    <t>TRIBUNALE*</t>
+  </si>
+  <si>
+    <t>UFFICIO POSTALE</t>
+  </si>
+  <si>
+    <t>ALTRA STR. SANITARIA</t>
+  </si>
+  <si>
+    <t>STR SOCIO SANITARIA</t>
+  </si>
+  <si>
+    <t>ACQUA</t>
+  </si>
+  <si>
+    <t>FERROVIA/METRO</t>
+  </si>
+  <si>
+    <t>IMPERVIO</t>
+  </si>
+  <si>
+    <t>IMPIANTO SCI</t>
+  </si>
+  <si>
+    <t>AMBULATORIO TERRITOR.</t>
+  </si>
+  <si>
+    <t>CENTRO DIURNO</t>
+  </si>
+  <si>
+    <t>BACINO</t>
+  </si>
+  <si>
+    <t>BANCHINA</t>
+  </si>
+  <si>
+    <t>ALPEGGIO</t>
+  </si>
+  <si>
+    <t>PISTA</t>
+  </si>
+  <si>
+    <t>PUNTO VACCINALE TER</t>
+  </si>
+  <si>
+    <t>COMUNITA'</t>
+  </si>
+  <si>
+    <t>CANALE</t>
+  </si>
+  <si>
+    <t>BIGLIETTERIA</t>
+  </si>
+  <si>
+    <t>BIVACCO</t>
+  </si>
+  <si>
+    <t>RISTORO</t>
+  </si>
+  <si>
+    <t>STUDIO MEDICO</t>
+  </si>
+  <si>
+    <t>CURE INTERMEDIE</t>
+  </si>
+  <si>
+    <t>CAVA</t>
+  </si>
+  <si>
+    <t>LINEA / BINARI</t>
+  </si>
+  <si>
+    <t>BOSCO</t>
+  </si>
+  <si>
+    <t>IMPIANTO RISALITA</t>
+  </si>
+  <si>
+    <t>HOSPICE</t>
+  </si>
+  <si>
+    <t>FIUME / TORRENTE</t>
+  </si>
+  <si>
+    <t>MEZZANINO</t>
+  </si>
+  <si>
+    <t>CAMPO</t>
+  </si>
+  <si>
+    <t>POST-ACUTI</t>
+  </si>
+  <si>
+    <t>LAGO</t>
+  </si>
+  <si>
+    <t>PASSAGGIO A LIVELLO</t>
+  </si>
+  <si>
+    <t>FUORI PISTA</t>
+  </si>
+  <si>
+    <t>POT (PRESIDI OSPEDALIERI TERRITORIALI)</t>
+  </si>
+  <si>
+    <t>POSTO POLIZIA</t>
+  </si>
+  <si>
+    <t>GHIACCIAIO</t>
+  </si>
+  <si>
+    <t>PUNTO VACCINALE</t>
+  </si>
+  <si>
+    <t>SCALE / ACCESSI</t>
+  </si>
+  <si>
+    <t>PARETE ROCCIOSA</t>
+  </si>
+  <si>
+    <t>RIABILITAZ. EXTRA H</t>
+  </si>
+  <si>
+    <t>STAZIONE</t>
+  </si>
+  <si>
+    <t>RIFUGIO</t>
+  </si>
+  <si>
+    <t>RSA / RSD</t>
+  </si>
+  <si>
+    <t>TRENO</t>
+  </si>
+  <si>
+    <t>SENTIERO</t>
+  </si>
+  <si>
+    <t>SPELEO / FORRA</t>
+  </si>
+  <si>
+    <t>SUB ACUTI</t>
   </si>
 </sst>
 </file>
@@ -538,7 +899,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -561,11 +922,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFC4C7C5"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFC4C7C5"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFC4C7C5"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFC4C7C5"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
@@ -578,6 +954,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1717,4 +2099,634 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87995D56-E79A-48A0-9CFF-FDF54FC4F50A}">
+  <dimension ref="A1:M26"/>
+  <sheetFormatPr defaultColWidth="58.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="29.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="47.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="23" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="21.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="L1" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="M1" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="L2" s="6" t="s">
+        <v>243</v>
+      </c>
+      <c r="M2" s="6" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>246</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="L3" s="6" t="s">
+        <v>249</v>
+      </c>
+      <c r="M3" s="6" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>252</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="L4" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="M4" s="6" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="L5" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="M5" s="6" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="H6" s="6"/>
+      <c r="I6" s="6" t="s">
+        <v>261</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>262</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="L6" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="M6" s="6"/>
+    </row>
+    <row r="7" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="L7" s="6" t="s">
+        <v>267</v>
+      </c>
+      <c r="M7" s="6"/>
+    </row>
+    <row r="8" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="H8" s="6"/>
+      <c r="I8" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="J8" s="6"/>
+      <c r="K8" s="6" t="s">
+        <v>269</v>
+      </c>
+      <c r="L8" s="6" t="s">
+        <v>270</v>
+      </c>
+      <c r="M8" s="6"/>
+    </row>
+    <row r="9" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="H9" s="6"/>
+      <c r="I9" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="J9" s="6"/>
+      <c r="K9" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="L9" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="M9" s="6"/>
+    </row>
+    <row r="10" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="H10" s="6"/>
+      <c r="I10" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="J10" s="6"/>
+      <c r="K10" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="L10" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="M10" s="6"/>
+    </row>
+    <row r="11" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="6"/>
+      <c r="B11" s="6" t="s">
+        <v>216</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="H11" s="6"/>
+      <c r="I11" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="J11" s="6"/>
+      <c r="K11" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="L11" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="M11" s="6"/>
+    </row>
+    <row r="12" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="6"/>
+      <c r="B12" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
+      <c r="H12" s="6"/>
+      <c r="I12" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="J12" s="6"/>
+      <c r="K12" s="6"/>
+      <c r="L12" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="M12" s="6"/>
+    </row>
+    <row r="13" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="6"/>
+      <c r="B13" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
+      <c r="H13" s="6"/>
+      <c r="I13" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="J13" s="6"/>
+      <c r="K13" s="6"/>
+      <c r="L13" s="6"/>
+      <c r="M13" s="6"/>
+    </row>
+    <row r="14" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="6"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="6"/>
+    </row>
+    <row r="15" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="6"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
+      <c r="G15" s="6"/>
+    </row>
+    <row r="16" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="6"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6" t="s">
+        <v>224</v>
+      </c>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="6"/>
+    </row>
+    <row r="17" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="6"/>
+      <c r="B17" s="6"/>
+      <c r="C17" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="D17" s="6"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="6"/>
+    </row>
+    <row r="18" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="6"/>
+      <c r="B18" s="6"/>
+      <c r="C18" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
+      <c r="G18" s="6"/>
+    </row>
+    <row r="19" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="6"/>
+      <c r="B19" s="6"/>
+      <c r="C19" s="6" t="s">
+        <v>227</v>
+      </c>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="6"/>
+    </row>
+    <row r="20" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="6"/>
+      <c r="B20" s="6"/>
+      <c r="C20" s="6" t="s">
+        <v>228</v>
+      </c>
+      <c r="D20" s="6"/>
+      <c r="E20" s="6"/>
+      <c r="F20" s="6"/>
+      <c r="G20" s="6"/>
+    </row>
+    <row r="21" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="6"/>
+      <c r="B21" s="6"/>
+      <c r="C21" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="D21" s="6"/>
+      <c r="E21" s="6"/>
+      <c r="F21" s="6"/>
+      <c r="G21" s="6"/>
+    </row>
+    <row r="22" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="6"/>
+      <c r="B22" s="6"/>
+      <c r="C22" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="D22" s="6"/>
+      <c r="E22" s="6"/>
+      <c r="F22" s="6"/>
+      <c r="G22" s="6"/>
+    </row>
+    <row r="23" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="6"/>
+      <c r="B23" s="6"/>
+      <c r="C23" s="6" t="s">
+        <v>230</v>
+      </c>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6"/>
+      <c r="F23" s="6"/>
+      <c r="G23" s="6"/>
+    </row>
+    <row r="24" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="6"/>
+      <c r="B24" s="6"/>
+      <c r="C24" s="6" t="s">
+        <v>231</v>
+      </c>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="6"/>
+      <c r="G24" s="6"/>
+    </row>
+    <row r="25" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="6"/>
+      <c r="B25" s="6"/>
+      <c r="C25" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="D25" s="6"/>
+      <c r="E25" s="6"/>
+      <c r="F25" s="6"/>
+      <c r="G25" s="6"/>
+    </row>
+    <row r="26" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="6"/>
+      <c r="B26" s="6"/>
+      <c r="C26" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="D26" s="6"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="6"/>
+      <c r="G26" s="6"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>